<commit_message>
bulk excel uploading successsfulll
</commit_message>
<xml_diff>
--- a/assets/28 entry testbed.xlsx
+++ b/assets/28 entry testbed.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Non Office\Dev Space\AppDev\kohatian_foundation\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB52D16F-26F7-4578-975C-BB8004E987CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90EA253E-5B63-46F7-B35B-F12411876D6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="15300" windowHeight="7785" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
   <si>
     <t>House</t>
   </si>
@@ -67,6 +67,12 @@
   </si>
   <si>
     <t>Charsadda</t>
+  </si>
+  <si>
+    <t>AloKan</t>
+  </si>
+  <si>
+    <t>Karak</t>
   </si>
 </sst>
 </file>
@@ -393,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
@@ -468,6 +474,23 @@
         <v>123456888</v>
       </c>
     </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2899</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5">
+        <v>564879123</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>